<commit_message>
Remove local paths and author names from the jar and the spreadsheets
The interview tool carried the absolute path of a local working directory as
the default root of its offline experiment parameters; it now defaults to the
working directory, and the jar is rebuilt from otherwise unchanged sources.
The three spreadsheets no longer record an author or the path they were
saved under; their cell data are unchanged.
</commit_message>
<xml_diff>
--- a/Artifact/llm_hockey/Interview with LLM Oracle.xlsx
+++ b/Artifact/llm_hockey/Interview with LLM Oracle.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\freem\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159F651D-6937-458C-8A9D-85C4FAF5EC36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="737" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>